<commit_message>
fix: improve date matching by day-of-year and fuzzy vehicle matching
</commit_message>
<xml_diff>
--- a/test_kilometraje.xlsx
+++ b/test_kilometraje.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:S44"/>
+  <dimension ref="A3:S199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="3"/>
@@ -1083,6 +1083,174 @@
         <v/>
       </c>
     </row>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125">
+      <c r="D125" t="n">
+        <v>114.962</v>
+      </c>
+      <c r="E125" t="n">
+        <v>0</v>
+      </c>
+      <c r="F125" t="n">
+        <v>28</v>
+      </c>
+      <c r="G125" t="n">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>